<commit_message>
docs: VOX photo-montage design system + EP01 storyboard v2
- MontageScene実装指示書 v1 (VOX): 写真モンタージュ基盤。生成AI動画を減らし
  静止画(Gemini/PD)をcrop/grade/KenBurns/合成で映像化。collage背景+labelBox追加
- VOXルック テンプレA〜D + MNT検証シーン(コラージュ)スタイルフレーム
- チャンネル設計書 改訂v4.4: 素材ソース優先を『モンタージュ優先・生成AI動画は最後、
  生成AI静止画は主力素材』へ再定義。琥珀#E8A33D追加・KenBurns標準化
- Remotionパターンカタログ v1: 登録型/コンポジション/モーション文法の再利用台帳
- 第1回コンテ表v2 (84カット/台本v2.1準拠) + 生成スクリプト。C33をcollageへ再タグ
- リポジトリ整理指示書 v1
- AGENTS.md ドキュメント地図に上記を追加

Remotion実装コード(Codex作業中)は本コミットに含めない。
</commit_message>
<xml_diff>
--- a/conte/第1回_コンテ表_v2.xlsx
+++ b/conte/第1回_コンテ表_v2.xlsx
@@ -4799,15 +4799,19 @@
           <t>バーネイズは、精神分析の医者に相談しました。返ってきた助言は、こうだったといいます。——たばこは、力の象徴だ。女性にとっては、自分の「たいまつ」になる。</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>助言は少し声を落として、内緒話の温度で</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>診察室のシルエット(AI生成・抽象寄り。人物特定できない画)</t>
+          <t>切り絵コラージュ(collage): Gemini静止画の医者/診察室を切り抜き、古紙・診療録テクスチャ板の上に配置。Ken Burnsで緩速。実在人物に似せない架空。生成AI動画は使わない(v4.4)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>生成AI(Runway/Gemini)</t>
+          <t>Remotion(モンタージュ)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4867,7 +4871,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>MNT_COLLAGE_DOCTOR</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">

</xml_diff>